<commit_message>
Updated USA model - 2025-09-12 22:32
</commit_message>
<xml_diff>
--- a/VerveStacks_USA/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
+++ b/VerveStacks_USA/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_USA\SubRES_Tmpl\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{CC6EE8F3-35D8-4C0E-B653-F8C150FAB212}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{8177A302-5DD8-4A3C-919F-E61663B9D91C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="7" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -9012,7 +9012,7 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C0859269-96E5-4EBF-BAB4-2C4C4F0CD346}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ACB7D6FA-0B37-4A1F-8FE4-3DE98FA316B7}">
   <dimension ref="B9:N119"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -13210,7 +13210,7 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DC829776-0CF7-4D84-91C6-D25659024241}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B57A7BCB-A5CF-4C11-8251-5F13ACAE7264}">
   <dimension ref="B9:AB286"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -30168,7 +30168,7 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5E1A06B4-EC05-4C86-8773-36A140D0F20D}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A1293FEF-DE1A-4DDC-BA91-4A33DA661BB9}">
   <dimension ref="B9:P73"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated USA model - 2025-09-12 23:16
</commit_message>
<xml_diff>
--- a/VerveStacks_USA/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
+++ b/VerveStacks_USA/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_USA\SubRES_Tmpl\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{8177A302-5DD8-4A3C-919F-E61663B9D91C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{C625C03D-C5E9-4D3E-A170-5057096FC93C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="7" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -9012,7 +9012,7 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ACB7D6FA-0B37-4A1F-8FE4-3DE98FA316B7}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2C6F098D-3EB2-4D69-AE85-8671E789F7C1}">
   <dimension ref="B9:N119"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -13210,7 +13210,7 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B57A7BCB-A5CF-4C11-8251-5F13ACAE7264}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E363F678-1826-457F-A250-99906835A666}">
   <dimension ref="B9:AB286"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -30168,7 +30168,7 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A1293FEF-DE1A-4DDC-BA91-4A33DA661BB9}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{443D687F-6FC1-4966-943F-1E482CC129C4}">
   <dimension ref="B9:P73"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated USA model - 2025-09-12 23:30
</commit_message>
<xml_diff>
--- a/VerveStacks_USA/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
+++ b/VerveStacks_USA/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_USA\SubRES_Tmpl\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{C625C03D-C5E9-4D3E-A170-5057096FC93C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{55B42716-8BEC-4C3C-9A8F-E01336B8B659}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="7" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -9012,7 +9012,7 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2C6F098D-3EB2-4D69-AE85-8671E789F7C1}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{441C32FF-12E3-403A-9971-F3117F6DB6AB}">
   <dimension ref="B9:N119"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -13210,7 +13210,7 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E363F678-1826-457F-A250-99906835A666}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{68EC361C-B6E7-4394-8D16-030E86B68593}">
   <dimension ref="B9:AB286"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -30168,7 +30168,7 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{443D687F-6FC1-4966-943F-1E482CC129C4}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D5BFE421-8B44-4164-9B24-2AF270F3B38C}">
   <dimension ref="B9:P73"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated USA model - 2025-09-12 23:44
</commit_message>
<xml_diff>
--- a/VerveStacks_USA/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
+++ b/VerveStacks_USA/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_USA\SubRES_Tmpl\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{55B42716-8BEC-4C3C-9A8F-E01336B8B659}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{8C2B40F8-AD15-4675-B4D2-444264F308B4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="7" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -9012,7 +9012,7 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{441C32FF-12E3-403A-9971-F3117F6DB6AB}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{122D0E28-339C-4116-9C6D-B5CB5D313BCC}">
   <dimension ref="B9:N119"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -13210,7 +13210,7 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{68EC361C-B6E7-4394-8D16-030E86B68593}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0FDA28D5-AEBA-4E30-92B9-4E6377B730E0}">
   <dimension ref="B9:AB286"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -30168,7 +30168,7 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D5BFE421-8B44-4164-9B24-2AF270F3B38C}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EF0C83C1-0098-4EC1-BBE0-669852664F23}">
   <dimension ref="B9:P73"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated USA model - 2025-09-13 01:27
</commit_message>
<xml_diff>
--- a/VerveStacks_USA/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
+++ b/VerveStacks_USA/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_USA\SubRES_Tmpl\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{8C2B40F8-AD15-4675-B4D2-444264F308B4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{8A424650-0821-4482-87C2-D5612552B0DC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="7" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -9012,7 +9012,7 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{122D0E28-339C-4116-9C6D-B5CB5D313BCC}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{02D2FE08-FF19-4D98-A756-998968EA2AAB}">
   <dimension ref="B9:N119"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -13210,7 +13210,7 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0FDA28D5-AEBA-4E30-92B9-4E6377B730E0}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{47809E32-AE94-49A7-86D2-8828E209FC5F}">
   <dimension ref="B9:AB286"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -30168,7 +30168,7 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EF0C83C1-0098-4EC1-BBE0-669852664F23}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E6A8E799-D320-4790-A6EF-39B6A78CAD8E}">
   <dimension ref="B9:P73"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated USA model - 2025-09-13 01:41
</commit_message>
<xml_diff>
--- a/VerveStacks_USA/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
+++ b/VerveStacks_USA/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_USA\SubRES_Tmpl\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{8A424650-0821-4482-87C2-D5612552B0DC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{FF2F7598-ACD5-4353-90BF-7BB1FBA40F09}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="7" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -9012,7 +9012,7 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{02D2FE08-FF19-4D98-A756-998968EA2AAB}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A27C565D-9C46-4C96-AB1B-262FF9C7B59F}">
   <dimension ref="B9:N119"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -13210,7 +13210,7 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{47809E32-AE94-49A7-86D2-8828E209FC5F}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D6A8BE6E-11D9-47E3-9A05-DFFE456E6A70}">
   <dimension ref="B9:AB286"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -30168,7 +30168,7 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E6A8E799-D320-4790-A6EF-39B6A78CAD8E}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{174FD076-6536-4531-88AD-788454223A93}">
   <dimension ref="B9:P73"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated USA model - 2025-09-13 09:03
</commit_message>
<xml_diff>
--- a/VerveStacks_USA/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
+++ b/VerveStacks_USA/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_USA\SubRES_Tmpl\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{FF2F7598-ACD5-4353-90BF-7BB1FBA40F09}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{D2C55F13-C88C-4860-A62E-67F04F598537}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="7" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -9012,7 +9012,7 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A27C565D-9C46-4C96-AB1B-262FF9C7B59F}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{729193DB-62BC-4CA8-98C4-907448DF5F4C}">
   <dimension ref="B9:N119"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -13210,7 +13210,7 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D6A8BE6E-11D9-47E3-9A05-DFFE456E6A70}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{66289F17-3DDD-4FEB-A0DF-EDA464CEC8EE}">
   <dimension ref="B9:AB286"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -30168,7 +30168,7 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{174FD076-6536-4531-88AD-788454223A93}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{17B94B80-9C90-49BC-8556-889A6DD8B6D7}">
   <dimension ref="B9:P73"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated USA model - 2025-09-13 09:45
</commit_message>
<xml_diff>
--- a/VerveStacks_USA/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
+++ b/VerveStacks_USA/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_USA\SubRES_Tmpl\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{D2C55F13-C88C-4860-A62E-67F04F598537}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{AEBF921E-3DED-4C54-90F6-586675FE8F5D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="7" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -9012,7 +9012,7 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{729193DB-62BC-4CA8-98C4-907448DF5F4C}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7FE263B6-8BC2-405A-84E9-1FF79022630E}">
   <dimension ref="B9:N119"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -13210,7 +13210,7 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{66289F17-3DDD-4FEB-A0DF-EDA464CEC8EE}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4DD6B64E-B48B-4273-8430-470E85A3AF08}">
   <dimension ref="B9:AB286"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -30168,7 +30168,7 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{17B94B80-9C90-49BC-8556-889A6DD8B6D7}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A4FB909D-5A2E-40A8-90EC-25EE2A7D75D3}">
   <dimension ref="B9:P73"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated USA model - 2025-09-13 16:51
</commit_message>
<xml_diff>
--- a/VerveStacks_USA/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
+++ b/VerveStacks_USA/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_USA\SubRES_Tmpl\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{AEBF921E-3DED-4C54-90F6-586675FE8F5D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{15CF3FF7-15EF-406C-94C7-00F48C12A7A2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="7" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -9012,7 +9012,7 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7FE263B6-8BC2-405A-84E9-1FF79022630E}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B9079522-CDA1-4115-8F9A-35644AAEF7BD}">
   <dimension ref="B9:N119"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -13210,7 +13210,7 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4DD6B64E-B48B-4273-8430-470E85A3AF08}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5DB32582-BAF4-4A5F-A6FA-7710236181F9}">
   <dimension ref="B9:AB286"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -30168,7 +30168,7 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A4FB909D-5A2E-40A8-90EC-25EE2A7D75D3}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F325FB98-D846-4B45-A297-25C7FFE7AB23}">
   <dimension ref="B9:P73"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated USA model - 2025-09-14 14:07
</commit_message>
<xml_diff>
--- a/VerveStacks_USA/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
+++ b/VerveStacks_USA/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_USA\SubRES_Tmpl\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{15CF3FF7-15EF-406C-94C7-00F48C12A7A2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{A4EBF827-B4A8-4D2F-9273-BB9F4669C069}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="7" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -9012,7 +9012,7 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B9079522-CDA1-4115-8F9A-35644AAEF7BD}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E9A23D24-ECB4-496A-92A4-E76FBA59BD61}">
   <dimension ref="B9:N119"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -13210,7 +13210,7 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5DB32582-BAF4-4A5F-A6FA-7710236181F9}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{28B4280A-73B6-4F52-AD1C-9E822C7497DE}">
   <dimension ref="B9:AB286"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -30168,7 +30168,7 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F325FB98-D846-4B45-A297-25C7FFE7AB23}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{24D5CD1C-EB56-449B-927E-8CBCD4EBAC26}">
   <dimension ref="B9:P73"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated USA model - 2025-12-12 16:07
</commit_message>
<xml_diff>
--- a/VerveStacks_USA/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
+++ b/VerveStacks_USA/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_USA\SubRES_Tmpl\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{F048C176-9281-4305-A735-BB6B13E6031A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{E62926E1-F18A-4A5D-B234-27296B0A884A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="6" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -8029,7 +8029,7 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D835E673-FE28-433A-BC22-0C405F9844E2}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{34A7C41C-69E5-4E90-82FC-33F523541089}">
   <dimension ref="B9:M149"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -12947,7 +12947,7 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AA974EC9-0E51-4966-8B9D-AF61D86B916B}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CE8DB4D0-A55F-4D31-AC92-792DCE16E7EB}">
   <dimension ref="B9:Z140"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -18084,7 +18084,7 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{85C35F28-2460-44B9-97B0-96ADB07F3396}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D2AB38A6-DBF1-477C-B745-8C7A16C4C76D}">
   <dimension ref="B9:P73"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>